<commit_message>
SEO: Optimierte Titel und Meta-Descriptions für alle verbleibenden Seiten
Behandlungen, Schulungen, Face Yoga, Über mich, Beauty News
und alle noch ausstehenden Blog-Artikel wurden mit optimierten
SEO-Titeln und Meta-Descriptions versehen. Excel-Übersicht aktualisiert.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEO_Uebersicht_kristin-schnoedt.xlsx
+++ b/SEO_Uebersicht_kristin-schnoedt.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +62,11 @@
       <color rgb="00999999"/>
       <sz val="9"/>
     </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +95,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="00ECDDE1"/>
         <bgColor rgb="00ECDDE1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -153,6 +161,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -632,14 +643,14 @@
           <t>Professionelle Gesichtsbehandlungen im Kosmetikstudio Auerbach: Klassische Behandlung, Gua Sha, Celluma Light Therapy, Microdermabrasion, Biomicroneedling. Individuell auf deine Haut abgestimmt.</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Gesichtsbehandlungen Auerbach | Kosmetikstudio Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Buccale Massage, Gua Sha, Microneedling &amp; mehr – Kosmetikbehandlungen in Auerbach für natürliche Hautverjüngung. Ohne Botox. Mit echten Ergebnissen.</t>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -669,14 +680,14 @@
           <t>Face Yoga, Cupping und PURVIDUAL Schulungen für Kosmetikerinnen. Außerdem: professionelle Website-Erstellung für Kosmetikstudios. Kristin Schnödt, 18 Jahre Erfahrung, Inhaberin PURVIDUAL.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Schulungen für Kosmetikerinnen | Face Yoga &amp; Cupping – Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Face Yoga, Cupping &amp; PURVIDUAL Schulungen für Kosmetikerinnen. Plus: professionelle Websites für Beauty Studios. Von Kristin Schnödt – 18+ Jahre Erfahrung.</t>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -706,14 +717,14 @@
           <t>Face Yoga mit Kristin Schnödt – natürliche Gesichtsverjüngung ohne Nadel und Skalpell. Entdecke die Methode, die deine Haut von innen strahlen lässt.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Face Yoga Online Kurs | Natürliche Hautverjüngung – Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Face Yoga Kurse mit Kristin Schnödt – natürliche Gesichtsverjüngung für Frauen ab 35. Online &amp; flexibel. Sichtbare Ergebnisse in wenigen Wochen. Jetzt entdecken.</t>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -743,14 +754,14 @@
           <t>Kristin Schnödt — Kosmetikerin aus Auerbach, Face Yoga Expertin und Gründerin von PURVIDUAL. Lerne mich kennen: meine Geschichte, meine Philosophie, mein Warum.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Kristin Schnödt – Kosmetikerin in Auerbach i.d.Opf.</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Kristin Schnödt – Spezialistin für natürliche Hautverjüngung in Auerbach. 18+ Jahre Erfahrung, anti-Botox, Gründerin von PURVIDUAL. Meine Geschichte &amp; Philosophie.</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -854,14 +865,14 @@
           <t>Wissen, Inspiration und Tipps rund um Face Yoga, Cupping, natürliche Hautpflege und ganzheitliche Schönheit — von Kristin Schnödt.</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Beauty News &amp; Tipps | Face Yoga, Hautpflege – Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Wissen &amp; Inspiration zu Face Yoga, Cupping, Microneedling und natürlicher Hautpflege – von Kosmetikerin Kristin Schnödt aus Auerbach.</t>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1002,14 +1013,14 @@
           <t>Kristin Schnödt sagt es direkt: Sie ist gegen Botox. Nicht ohne Grund. Hier erklärt sie, warum Face Yoga langfristig das Überzeugendere ist — ehrlich, ohne Moralisieren.</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Botox oder Face Yoga – was wirklich wirkt | Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Kristin Schnödt erklärt klar: Warum Face Yoga langfristig wirksamer ist als Botox – und was wirklich hinter beiden Methoden steckt. Ehrlich &amp; ohne Moralisieren.</t>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1039,14 +1050,14 @@
           <t>Dein Gesicht hat über 40 Muskeln — und die meisten trainieren wir nie. Kristin Schnödt zeigt dir 5 Face Yoga Übungen, die sie selbst jeden Morgen macht.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>5 Face Yoga Übungen für sofortige Wirkung | Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Dein Gesicht hat über 40 Muskeln – und die meisten schlafen. Kristin Schnödt zeigt 5 Face Yoga Übungen für zuhause, die sie täglich selbst macht.</t>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1113,14 +1124,14 @@
           <t>Gesichtscupping klingt erstmal ungewohnt — aber kaum eine Technik aktiviert Lymphfluss, Durchblutung und Bindegewebe so effektiv. Kristin Schnödt erklärt, warum sie es liebt.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Gesichtscupping – Was es ist &amp; warum es wirkt | Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Gesichtscupping aktiviert Lymphfluss, Durchblutung und Bindegewebe wie kaum eine andere Technik. Kristin Schnödt erklärt die Methode und warum sie täglich damit arbeitet.</t>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1150,14 +1161,14 @@
           <t>Ab 40 verlangsamt sich die Zellerneuerung, Kollagen nimmt ab und die Haut reagiert empfindlicher. Kristin Schnödt erklärt, was dahintersteckt — und wie du wirklich gegensteuern kannst.</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Haut ab 40 – was sich verändert &amp; was wirklich hilft | Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Ab 40 verlangsamt sich die Zellerneuerung, Kollagen nimmt ab. Kristin Schnödt erklärt, was hinter Hautveränderungen ab 40 steckt – und wie du wirklich gegensteuern kannst.</t>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1224,14 +1235,14 @@
           <t>Viele Kundinnen kommen mit 12-Schritt-Routinen zu mir — und gehen mit drei Produkten nach Hause. Kristin Schnödt erklärt, warum Vereinfachung oft die wirkungsvollste Entscheidung ist.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Warum weniger Pflege mehr bewirkt | Kristin Schnödt</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Viele kommen mit 12-Schritt-Routinen zu Kristin Schnödt – und gehen mit 3 Produkten nach Hause. Warum Vereinfachung in der Hautpflege oft das Wirksamste ist.</t>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>✅ Optimiert</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">

</xml_diff>